<commit_message>
html spitting out from data
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lee.cockcroft\Downloads\compress\react\dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FDD5E63-8424-44CC-95A3-FEA40BE86644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75350E26-FB25-4212-9341-93627C0BA0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5920" yWindow="2940" windowWidth="14400" windowHeight="8170" xr2:uid="{A8C7D3E3-6759-4B5C-A6D9-4D659D49D801}"/>
+    <workbookView xWindow="3645" yWindow="-17775" windowWidth="28800" windowHeight="15225" xr2:uid="{A8C7D3E3-6759-4B5C-A6D9-4D659D49D801}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>title</t>
   </si>
   <si>
-    <t>dd</t>
-  </si>
-  <si>
     <t>standardterms</t>
   </si>
   <si>
@@ -68,85 +65,44 @@
     <t>ribbon3bottom</t>
   </si>
   <si>
-    <t>terms</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;What is the promotion and how do I qualify?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;The Sun Vegas are offering players the chance to receive up to 70 free spins. Simply opt in, and receive 10 free spins on each day that you spend &amp;pound;10 on Better Wilds Valentines.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;When is the promotion?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;The promotion runs between 09.02.26 and 15.02.26.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;Who is eligible?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;The Sun Vegas registered players, who are UK residents, aged 18+ years old (registration and ID verification required) and have deposited &amp;pound;10 or more in the 28 days prior to the promotion ending.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;What will I receive?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;You can receive 10 free spins each day, which you must accept via a pop-up message. A maximum of 70 free spins can be issued during the promotional period.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Free spins can be used on Better Wilds Valentines.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;What do I need to wager before I can withdraw any winnings?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;You are required to wager your winnings 3 times on the selected slot. Your free spins will expire 7 days after they have been credited. If the wagering requirements have not been met by this time, any remaining free spins + pending winnings shall be removed. You are entitled to withdraw your real cash balance and winnings derived from your real cash balance at any time. However, if the wagering requirements are not completed then players will forfeit any remaining free spins and any pending winnings from the spins.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Free Spins and their wagering requirements can be found by visiting &amp;ldquo;My Account&amp;rdquo; from the Home Page, clicking &amp;ldquo;History&amp;rdquo; and then &amp;ldquo;Bonus History.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;How are my funds used?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Free spins can be used at any stage, prior to the expiry date. Your winnings from wagering with free spins will be attributed to &amp;ldquo;Pending Winnings&amp;rdquo;. When you have winnings and play a game on which you can use your free spins, you will wager funds in the following order:&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;ol&gt;</t>
-  </si>
-  <si>
-    <t>&lt;li&gt;Pending winnings &amp;ndash; from play with your free spins&lt;/li&gt;</t>
-  </si>
-  <si>
-    <t>&lt;li&gt;Any remaining spins/coins from the offer&lt;/li&gt;</t>
-  </si>
-  <si>
-    <t>&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&lt;strong&gt;Can I claim any other bonuses while this bonus is active on my account?&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;You may make use of any other promotion, however, wagering requirements must be met for each bonus separately and in the order the bonus was claimed.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>18++++++</t>
-  </si>
-  <si>
-    <t>ww</t>
-  </si>
-  <si>
-    <t>w</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
     <t>ribbon2top</t>
   </si>
   <si>
     <t>ribbon3top</t>
+  </si>
+  <si>
+    <t>to The Sun Vegas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGISTER </t>
+  </si>
+  <si>
+    <t>on selected games</t>
+  </si>
+  <si>
+    <t>DOUBLE YOUR DEPOSIT
+UP TO £300 PLUS</t>
+  </si>
+  <si>
+    <t>100 FREE SPINS</t>
+  </si>
+  <si>
+    <t>Deposit £10</t>
+  </si>
+  <si>
+    <t>for 100% bonus match</t>
+  </si>
+  <si>
+    <t>GET 100 FREE SPINS</t>
+  </si>
+  <si>
+    <t>18+. New customers only. Min deposit £10 for 100% deposit match bonus up to £300 (wager bonus 10x within 30 days on selected games) and 100 Free Spins (wager winnings 10x within 7 days on selected games). Accept bonus &amp; free spins within 48hrs. Debit cards only. Offer ends 30.04.26.</t>
+  </si>
+  <si>
+    <t>100% deposit matrch and free spins</t>
+  </si>
+  <si>
+    <t>bigbass</t>
   </si>
 </sst>
 </file>
@@ -182,8 +138,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,189 +477,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A71F159-57F8-43B4-9BB8-6283AACB64F3}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6328125" customWidth="1"/>
+    <col min="4" max="4" width="27.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.7265625" customWidth="1"/>
-    <col min="10" max="11" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="67.453125" customWidth="1"/>
     <col min="15" max="15" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
       <c r="K1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
+        <v>21</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L10" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L13" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L14" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="12:12" x14ac:dyDescent="0.35">
-      <c r="L21" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>